<commit_message>
Wire B21 underdrain into ds/Af/t_vid formulas
When B21=0 (no underdrain), exclude gravel voids from ds and use
infiltration-only drawdown; Couches/Scenarios/Methode/README follow B21.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/bioretention/Bioretention_Dimensionnement_v1.xlsx
+++ b/engineering/drainage-design/bioretention/Bioretention_Dimensionnement_v1.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -803,14 +803,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1 = avec underdrain; 0 = infiltration seule</t>
+          <t>1 = underdrain (dr compte dans ds; tp = ennoiement). 0 = infiltration seule (dr exclu; tp = profil)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>3) Résultats (formules live)</t>
+          <t>3) Résultats (formules live — dépendent de B21)</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Vcap = η × C × (Rd/1000) × Ad</t>
+          <t>Vcap = η × C × (Rd/1000) × Ad  (indépendant de B21)</t>
         </is>
       </c>
     </row>
@@ -837,12 +837,12 @@
         </is>
       </c>
       <c r="B25" s="10">
-        <f>B12+B17*B18+B13*B14+B15*B16</f>
+        <f>IF(B21=1,B12+B17*B18+B13*B14+B15*B16,B12+B17*B18+B13*B14)</f>
         <v/>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ds = dp + dm·nm + df·nf + dr·nr</t>
+          <t>B21=1: ds=dp+dm·nm+df·nf+dr·nr · B21=0: sans dr·nr (pas de crédit réservoir drainé)</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Af = Vcap / ds</t>
+          <t>Af = Vcap / ds  → augmente si B21=0 (ds plus petit)</t>
         </is>
       </c>
     </row>
@@ -881,87 +881,98 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Temps de vidange de l'ennoiement tp (h)</t>
+          <t>Temps de vidange gouvernant t_vid (h)</t>
         </is>
       </c>
       <c r="B28" s="11">
-        <f>IF(B19&lt;=0,"f'=0",B12/(B19/1000))</f>
+        <f>IF(B19&lt;=0,"f'=0",IF(B21=1,B12/(B19/1000),(B12+B13*B14)/(B19/1000)))</f>
         <v/>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>tp = dp / (f'/1000) — ennoiement de surface</t>
+          <t>B21=1: t=dp/(f'/1000) · B21=0: t=(dp+df·nf)/(f'/1000) infiltration seule</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Temps approximatif média→réservoir tm (h)</t>
+          <t>Temps média (+gravier si drain) tm (h)</t>
         </is>
       </c>
       <c r="B29" s="11">
-        <f>IF(B19&lt;=0,"f'=0",(B13*B14+B15*B16)/(B19/1000))</f>
+        <f>IF(B19&lt;=0,"f'=0",(B13*B14+IF(B21=1,B15*B16,0))/(B19/1000))</f>
         <v/>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Approximatif: (df·nf + dr·nr) / (f'/1000)</t>
+          <t>(df·nf + B21·dr·nr) / (f'/1000)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Vidange OK vs t_max?</t>
+          <t>Mode hydraulique</t>
         </is>
       </c>
       <c r="B30" s="12">
-        <f>IF(OR(B28="f'=0",B28=""),"",IF(B28&lt;=B20,"OUI — tp ≤ t_max","NON — augmenter Af, dp↓ ou f'"))</f>
+        <f>IF(B21=1,"Avec sous-drain (SWMM Drain coeff &gt; 0)","Sans sous-drain (SWMM Drain coeff = 0)")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Longueur indicative L si largeur = 3 m</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n">
-        <v>3</v>
+          <t>Vidange OK vs t_max?</t>
+        </is>
+      </c>
+      <c r="B31" s="12">
+        <f>IF(OR(B28="f'=0",B28=""),"",IF(B28&lt;=B20,"OUI — t_vid ≤ t_max","NON — ↑Af, ↓dp, ↑f' ou ajouter drain"))</f>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Longueur L (m) pour largeur B31</t>
-        </is>
-      </c>
-      <c r="B32" s="11">
-        <f>IF(B31&lt;=0,"",B26/B31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+          <t>Longueur indicative L si largeur = 3 m</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Longueur L (m) pour largeur B32</t>
+        </is>
+      </c>
+      <c r="B33" s="11">
+        <f>IF(B32&lt;=0,"",B26/B32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Message produit</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Livrable: Af + Vcap + tp. Ce n'est PAS un design final CSA W200 — valider géotechnique (f'), plantation, prétraitement, trop-plein et exigences municipales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36"/>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Livrable: Af + Vcap + t_vid. B21 change ds/Af/t_vid. Pas un design final CSA W200 — valider f', plantation, prétraitement, trop-plein, municipalité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F3"/>
-    <mergeCell ref="A35:F36"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A36:F37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -991,12 +1002,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Af liée à Parametres!B26. Volumes = Af × profondeur × porosité (stockage).</t>
-        </is>
-      </c>
-    </row>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Af = Parametres!B26. Stockage = Af × profondeur × porosité. Gravier crédité seulement si Parametres!B21=1 (sous-drain).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -1095,7 +1107,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Réservoir / gravier</t>
+          <t>Réservoir / gravier (×B21)</t>
         </is>
       </c>
       <c r="B8" s="10">
@@ -1107,18 +1119,18 @@
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>Parametres!$B$26*B8*C8</f>
+        <f>Parametres!$B$21*Parametres!$B$26*B8*C8</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>Parametres!$B$26*B8</f>
+        <f>Parametres!$B$21*Parametres!$B$26*B8</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Stockage total (m3)</t>
+          <t>Stockage total crédité (m3)</t>
         </is>
       </c>
       <c r="B10" s="9">
@@ -1138,11 +1150,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>≈ 0 si Af = Vcap/ds</t>
+          <t>≈ 0 si Af = Vcap/ds (gravier exclu quand B21=0)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1154,7 +1169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1197,7 +1212,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>tp (h)</t>
+          <t>t_vid (h)</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -1219,7 +1234,7 @@
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>IF(Parametres!$B$19&lt;=0,0,Parametres!$B$12/(Parametres!$B$19/1000))</f>
+        <f>IF(Parametres!$B$19&lt;=0,0,IF(Parametres!$B$21=1,Parametres!$B$12/(Parametres!$B$19/1000),(Parametres!$B$12+Parametres!$B$13*Parametres!$B$14)/(Parametres!$B$19/1000)))</f>
         <v/>
       </c>
       <c r="E6" s="15">
@@ -1240,7 +1255,7 @@
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>IF(Parametres!$B$19&lt;=0,0,Parametres!$B$12/(Parametres!$B$19/1000))</f>
+        <f>IF(Parametres!$B$19&lt;=0,0,IF(Parametres!$B$21=1,Parametres!$B$12/(Parametres!$B$19/1000),(Parametres!$B$12+Parametres!$B$13*Parametres!$B$14)/(Parametres!$B$19/1000)))</f>
         <v/>
       </c>
       <c r="E7" s="15">
@@ -1261,7 +1276,7 @@
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>IF(Parametres!$B$19&lt;=0,0,Parametres!$B$12/(Parametres!$B$19/1000))</f>
+        <f>IF(Parametres!$B$19&lt;=0,0,IF(Parametres!$B$21=1,Parametres!$B$12/(Parametres!$B$19/1000),(Parametres!$B$12+Parametres!$B$13*Parametres!$B$14)/(Parametres!$B$19/1000)))</f>
         <v/>
       </c>
       <c r="E8" s="15">
@@ -1270,14 +1285,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Note: tp dépend de dp et f', pas de Rd — colonne D identique par scénario.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Note: t_vid dépend de B21, dp, f' (et df·nf si B21=0) — pas de Rd. Colonne D identique par scénario. Af change avec ds(B21).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A11:E12"/>
     <mergeCell ref="A2:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1290,7 +1307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1319,143 +1336,188 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Formules:</t>
+          <t>Formules (B21 = sous-drain 1/0):</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Vcap = η × C × (Rd/1000) × Ad</t>
+          <t xml:space="preserve">  Vcap = η × C × (Rd/1000) × Ad     (indépendant de B21)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ds   = dp + dm·nm + df·nf + dr·nr</t>
+          <t xml:space="preserve">  B21=1: ds = dp + dm·nm + df·nf + dr·nr</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Af   = Vcap / ds</t>
+          <t xml:space="preserve">  B21=0: ds = dp + dm·nm + df·nf          (pas de crédit réservoir drainé)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  tp   = dp / (f'/1000)   avec f' en mm/h</t>
+          <t xml:space="preserve">  Af   = Vcap / ds</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B21=1: t_vid = dp / (f'/1000)            (vidange d'ennoiement)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hypothèses simplifiées (à déclarer dans la note de calcul):</t>
+          <t xml:space="preserve">  B21=0: t_vid = (dp + df·nf) / (f'/1000)  (infiltration seule)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Volume de captage type « qualité d'eau / petite pluie » (Rd souvent 25 mm).</t>
+          <t xml:space="preserve">  tm   = (df·nf + B21·dr·nr) / (f'/1000)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Stockage = ennoiement + vides média + vides réservoir (porosités effectives).</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Vidange de surface basée sur f' de conception (essai in situ ÷ facteur de sécurité).</t>
+          <t>Lien SWMM LID (Drain tab):</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Sous-drain: case B21 informative; un design CSA W200 détaille diamètre, pente, IWS, etc.</t>
+          <t xml:space="preserve">  B21=1 → Drain Coefficient &gt; 0 (underdrain actif)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B21=0 → Drain Coefficient = 0 (infiltration seule)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Références à citer (ne pas copier le texte normatif):</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • CSA W200:18 (R2023) Design of bioretention systems</t>
+          <t>Hypothèses simplifiées (à déclarer dans la note de calcul):</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • STEP / Sustainable Technologies — Bioretention: Sizing (guide LID)</t>
+          <t xml:space="preserve">  • Volume de captage type « qualité d'eau / petite pluie » (Rd souvent 25 mm).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Exigences municipales locales (Montréal / arrondissement / schéma)</t>
+          <t xml:space="preserve">  • Stockage crédité = ennoiement + vides média (+ vides gravier seulement si B21=1).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Vidange basée sur f' de conception (essai in situ ÷ facteur de sécurité).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Prochaines versions possibles:</t>
+          <t xml:space="preserve">  • B21 pilote ds / Af / t_vid; un design CSA W200 détaille diamètre, pente, IWS, etc.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  v1.1 hydrogramme + bypass</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  v1.2 prétraitement (fosse à sédiments)</t>
+          <t>Références à citer (ne pas copier le texte normatif):</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  v1.3 plantation / sel de voirie (climat froid QC)</t>
+          <t xml:space="preserve">  • CSA W200:18 (R2023) Design of bioretention systems</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • STEP / Sustainable Technologies — Bioretention: Sizing (guide LID)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Exigences municipales locales (Montréal / arrondissement / schéma)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Prochaines versions possibles:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  v1.1 hydrogramme + bypass</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  v1.2 prétraitement (fosse à sédiments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  v1.3 plantation / sel de voirie (climat froid QC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Regénérer: python3 build_bioretention_excel.py</t>
         </is>

</xml_diff>